<commit_message>
Added more documentation; more comments and cleanup in mcts_multiple_expansion.py
</commit_message>
<xml_diff>
--- a/docs/Papers/iot_sensor_papers.xlsx
+++ b/docs/Papers/iot_sensor_papers.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roman\PycharmProjects\bachelorThesis\Results\Papers\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roman\PycharmProjects\bachelorThesis\docs\Papers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A90AFCA7-D28A-4F8B-8F78-4603924D1831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8C8A33-78EB-4A9D-963D-5E801F562BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5400" yWindow="-5385" windowWidth="18240" windowHeight="29040" xr2:uid="{4BB29169-61E1-4DE9-82FD-04B604469E05}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{4BB29169-61E1-4DE9-82FD-04B604469E05}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
   <si>
     <t>Reference</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>Rusu, C. A., Melhem, R., &amp; Mosse, D. (2003). Maximizing the system value while satisfying time and energy constraints. IBM Journal of Research and Development, 47(5.6), 689-702.</t>
+  </si>
+  <si>
+    <t>MICAz Datasheet</t>
   </si>
 </sst>
 </file>
@@ -518,7 +521,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E626032-7D24-48C2-9499-FD2EFC8C1634}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="68.85546875" customWidth="1"/>
@@ -773,6 +776,17 @@
       </c>
       <c r="D24" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D25" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -800,8 +814,9 @@
     <hyperlink ref="A22" r:id="rId21" xr:uid="{5F3BCD90-0B65-4DAA-A665-58BA38162C76}"/>
     <hyperlink ref="A23" r:id="rId22" xr:uid="{8C5183D0-E4C9-458B-8558-4109679B5E0B}"/>
     <hyperlink ref="A24" r:id="rId23" xr:uid="{503B01CC-4035-42EB-B635-F6BC7DB64AB7}"/>
+    <hyperlink ref="A25" r:id="rId24" display="MicaZ Datasheet" xr:uid="{53FC7695-21E4-4BCA-A726-ADDD3AA4E449}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId24"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId25"/>
 </worksheet>
 </file>
</xml_diff>